<commit_message>
Add a future-date check and derive the review data once
DT-FUT (check type future_date) flags dates later than the data cut,
the latest availability date in the extract. run_checks reuses the
derived snapshot from review_data instead of deriving again.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/studies/example/check_spec.xlsx
+++ b/studies/example/check_spec.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="182">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -157,6 +157,27 @@
     <t xml:space="preserve">warning</t>
   </si>
   <si>
+    <t xml:space="preserve">DT-FUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date after the data cut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A collected date later than the extract date, usually a typing error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">future_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data management</t>
+  </si>
+  <si>
     <t xml:space="preserve">AE-COD</t>
   </si>
   <si>
@@ -166,12 +187,6 @@
     <t xml:space="preserve">Adverse event entered but not yet coded</t>
   </si>
   <si>
-    <t xml:space="preserve">Data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data</t>
-  </si>
-  <si>
     <t xml:space="preserve">missing_value</t>
   </si>
   <si>
@@ -181,9 +196,6 @@
     <t xml:space="preserve">Awaiting coding</t>
   </si>
   <si>
-    <t xml:space="preserve">data management</t>
-  </si>
-  <si>
     <t xml:space="preserve">DS-DISC</t>
   </si>
   <si>
@@ -463,6 +475,24 @@
     <t xml:space="preserve">Missed visit: FORM SV, FIELD VISDAT, PARAMS statuses=Missed; not_done=VISND == Yes</t>
   </si>
   <si>
+    <t xml:space="preserve">Dates later than the data cut (the extract date), usually typing errors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Form; blank for every form</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date fields; blank for every date field</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">exclude=fields to leave out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date after the data cut: FORM and FIELD blank</t>
+  </si>
+  <si>
     <t xml:space="preserve">Values outside a range</t>
   </si>
   <si>
@@ -482,9 +512,6 @@
   </si>
   <si>
     <t xml:space="preserve">Field(s), comma-separated</t>
-  </si>
-  <si>
-    <t xml:space="preserve"/>
   </si>
   <si>
     <t xml:space="preserve">AE not coded: FORM AE, FIELD AEDECOD</t>
@@ -1123,22 +1150,16 @@
       <c r="F5" t="s">
         <v>52</v>
       </c>
-      <c r="G5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" t="s">
-        <v>53</v>
-      </c>
+      <c r="G5"/>
+      <c r="H5"/>
       <c r="I5"/>
       <c r="J5"/>
-      <c r="K5" t="s">
-        <v>54</v>
-      </c>
+      <c r="K5"/>
       <c r="L5" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="M5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="N5" t="s">
         <v>29</v>
@@ -1155,41 +1176,39 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" t="s">
         <v>56</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F6" t="s">
         <v>57</v>
       </c>
-      <c r="C6" t="s">
+      <c r="G6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" t="s">
         <v>58</v>
       </c>
-      <c r="D6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" t="s">
-        <v>60</v>
-      </c>
-      <c r="H6" t="s">
-        <v>61</v>
-      </c>
-      <c r="I6" t="s">
-        <v>62</v>
-      </c>
+      <c r="I6"/>
       <c r="J6"/>
       <c r="K6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L6" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="M6" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="N6" t="s">
         <v>29</v>
@@ -1206,16 +1225,16 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D7" t="s">
         <v>63</v>
-      </c>
-      <c r="B7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D7" t="s">
-        <v>66</v>
       </c>
       <c r="E7" t="s">
         <v>21</v>
@@ -1224,17 +1243,17 @@
         <v>22</v>
       </c>
       <c r="G7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="H7" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="J7"/>
       <c r="K7" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="L7" t="s">
         <v>46</v>
@@ -1257,34 +1276,36 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B8" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D8" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E8" t="s">
         <v>21</v>
       </c>
       <c r="F8" t="s">
-        <v>75</v>
+        <v>22</v>
       </c>
       <c r="G8" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="H8" t="s">
-        <v>77</v>
-      </c>
-      <c r="I8"/>
-      <c r="J8" t="s">
-        <v>78</v>
-      </c>
-      <c r="K8"/>
+        <v>72</v>
+      </c>
+      <c r="I8" t="s">
+        <v>73</v>
+      </c>
+      <c r="J8"/>
+      <c r="K8" t="s">
+        <v>74</v>
+      </c>
       <c r="L8" t="s">
         <v>46</v>
       </c>
@@ -1306,28 +1327,28 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" t="s">
         <v>79</v>
       </c>
-      <c r="B9" t="s">
+      <c r="G9" t="s">
         <v>80</v>
       </c>
-      <c r="C9" t="s">
+      <c r="H9" t="s">
         <v>81</v>
-      </c>
-      <c r="D9" t="s">
-        <v>74</v>
-      </c>
-      <c r="E9" t="s">
-        <v>51</v>
-      </c>
-      <c r="F9" t="s">
-        <v>75</v>
-      </c>
-      <c r="G9" t="s">
-        <v>76</v>
-      </c>
-      <c r="H9" t="s">
-        <v>77</v>
       </c>
       <c r="I9"/>
       <c r="J9" t="s">
@@ -1338,7 +1359,7 @@
         <v>46</v>
       </c>
       <c r="M9" t="s">
-        <v>83</v>
+        <v>21</v>
       </c>
       <c r="N9" t="s">
         <v>29</v>
@@ -1355,39 +1376,39 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" t="s">
         <v>84</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>85</v>
       </c>
-      <c r="C10" t="s">
-        <v>86</v>
-      </c>
       <c r="D10" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E10" t="s">
         <v>51</v>
       </c>
       <c r="F10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H10" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="I10"/>
       <c r="J10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="K10"/>
       <c r="L10" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="M10" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="N10" t="s">
         <v>29</v>
@@ -1413,32 +1434,30 @@
         <v>90</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="E11" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F11" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="G11" t="s">
+        <v>80</v>
+      </c>
+      <c r="H11" t="s">
+        <v>81</v>
+      </c>
+      <c r="I11"/>
+      <c r="J11" t="s">
         <v>91</v>
       </c>
-      <c r="H11" t="s">
-        <v>92</v>
-      </c>
-      <c r="I11" t="s">
-        <v>93</v>
-      </c>
-      <c r="J11"/>
-      <c r="K11" t="s">
-        <v>94</v>
-      </c>
+      <c r="K11"/>
       <c r="L11" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="M11" t="s">
-        <v>28</v>
+        <v>87</v>
       </c>
       <c r="N11" t="s">
         <v>29</v>
@@ -1447,21 +1466,21 @@
         <v>30</v>
       </c>
       <c r="P11" t="s">
-        <v>95</v>
+        <v>31</v>
       </c>
       <c r="Q11" t="s">
-        <v>96</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B12" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C12" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="D12" t="s">
         <v>20</v>
@@ -1473,20 +1492,20 @@
         <v>22</v>
       </c>
       <c r="G12" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="H12" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="I12" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="J12"/>
       <c r="K12" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="L12" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="M12" t="s">
         <v>28</v>
@@ -1498,24 +1517,24 @@
         <v>30</v>
       </c>
       <c r="P12" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="Q12" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
+        <v>101</v>
+      </c>
+      <c r="B13" t="s">
         <v>102</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>103</v>
       </c>
-      <c r="C13" t="s">
-        <v>104</v>
-      </c>
       <c r="D13" t="s">
-        <v>105</v>
+        <v>20</v>
       </c>
       <c r="E13" t="s">
         <v>21</v>
@@ -1524,23 +1543,23 @@
         <v>22</v>
       </c>
       <c r="G13" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="H13" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="I13" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="J13"/>
       <c r="K13" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="L13" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="M13" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="N13" t="s">
         <v>29</v>
@@ -1549,47 +1568,49 @@
         <v>30</v>
       </c>
       <c r="P13" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="Q13" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
+        <v>106</v>
+      </c>
+      <c r="B14" t="s">
+        <v>107</v>
+      </c>
+      <c r="C14" t="s">
+        <v>108</v>
+      </c>
+      <c r="D14" t="s">
+        <v>109</v>
+      </c>
+      <c r="E14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G14" t="s">
         <v>110</v>
       </c>
-      <c r="B14" t="s">
+      <c r="H14" t="s">
         <v>111</v>
       </c>
-      <c r="C14" t="s">
+      <c r="I14" t="s">
         <v>112</v>
       </c>
-      <c r="D14" t="s">
-        <v>50</v>
-      </c>
-      <c r="E14" t="s">
-        <v>51</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="J14"/>
+      <c r="K14" t="s">
         <v>113</v>
       </c>
-      <c r="G14" t="s">
-        <v>76</v>
-      </c>
-      <c r="H14"/>
-      <c r="I14" t="s">
-        <v>114</v>
-      </c>
-      <c r="J14" t="s">
-        <v>115</v>
-      </c>
-      <c r="K14"/>
       <c r="L14" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="M14" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="N14" t="s">
         <v>29</v>
@@ -1598,21 +1619,21 @@
         <v>30</v>
       </c>
       <c r="P14" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="Q14" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
+        <v>114</v>
+      </c>
+      <c r="B15" t="s">
+        <v>115</v>
+      </c>
+      <c r="C15" t="s">
         <v>116</v>
-      </c>
-      <c r="B15" t="s">
-        <v>117</v>
-      </c>
-      <c r="C15" t="s">
-        <v>118</v>
       </c>
       <c r="D15" t="s">
         <v>50</v>
@@ -1621,14 +1642,14 @@
         <v>51</v>
       </c>
       <c r="F15" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="G15" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H15"/>
       <c r="I15" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="J15" t="s">
         <v>119</v>
@@ -1638,7 +1659,7 @@
         <v>46</v>
       </c>
       <c r="M15" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="N15" t="s">
         <v>29</v>
@@ -1647,10 +1668,10 @@
         <v>30</v>
       </c>
       <c r="P15" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="Q15" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16">
@@ -1664,30 +1685,30 @@
         <v>122</v>
       </c>
       <c r="D16" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="E16" t="s">
         <v>51</v>
       </c>
       <c r="F16" t="s">
+        <v>117</v>
+      </c>
+      <c r="G16" t="s">
+        <v>80</v>
+      </c>
+      <c r="H16"/>
+      <c r="I16" t="s">
+        <v>118</v>
+      </c>
+      <c r="J16" t="s">
         <v>123</v>
-      </c>
-      <c r="G16" t="s">
-        <v>67</v>
-      </c>
-      <c r="H16" t="s">
-        <v>124</v>
-      </c>
-      <c r="I16"/>
-      <c r="J16" t="s">
-        <v>125</v>
       </c>
       <c r="K16"/>
       <c r="L16" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="M16" t="s">
-        <v>83</v>
+        <v>53</v>
       </c>
       <c r="N16" t="s">
         <v>29</v>
@@ -1696,49 +1717,47 @@
         <v>30</v>
       </c>
       <c r="P16" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="Q16" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
+        <v>124</v>
+      </c>
+      <c r="B17" t="s">
+        <v>125</v>
+      </c>
+      <c r="C17" t="s">
         <v>126</v>
       </c>
-      <c r="B17" t="s">
-        <v>127</v>
-      </c>
-      <c r="C17" t="s">
-        <v>128</v>
-      </c>
       <c r="D17" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E17" t="s">
         <v>51</v>
       </c>
       <c r="F17" t="s">
+        <v>127</v>
+      </c>
+      <c r="G17" t="s">
+        <v>71</v>
+      </c>
+      <c r="H17" t="s">
+        <v>128</v>
+      </c>
+      <c r="I17"/>
+      <c r="J17" t="s">
         <v>129</v>
-      </c>
-      <c r="G17" t="s">
-        <v>76</v>
-      </c>
-      <c r="H17" t="s">
-        <v>77</v>
-      </c>
-      <c r="I17" t="s">
-        <v>130</v>
-      </c>
-      <c r="J17" t="s">
-        <v>131</v>
       </c>
       <c r="K17"/>
       <c r="L17" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="M17" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="N17" t="s">
         <v>29</v>
@@ -1747,36 +1766,40 @@
         <v>30</v>
       </c>
       <c r="P17" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="Q17" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
+        <v>130</v>
+      </c>
+      <c r="B18" t="s">
+        <v>131</v>
+      </c>
+      <c r="C18" t="s">
         <v>132</v>
       </c>
-      <c r="B18" t="s">
-        <v>133</v>
-      </c>
-      <c r="C18" t="s">
-        <v>134</v>
-      </c>
       <c r="D18" t="s">
-        <v>50</v>
+        <v>78</v>
       </c>
       <c r="E18" t="s">
         <v>51</v>
       </c>
       <c r="F18" t="s">
-        <v>113</v>
+        <v>133</v>
       </c>
       <c r="G18" t="s">
-        <v>91</v>
-      </c>
-      <c r="H18"/>
-      <c r="I18"/>
+        <v>80</v>
+      </c>
+      <c r="H18" t="s">
+        <v>81</v>
+      </c>
+      <c r="I18" t="s">
+        <v>134</v>
+      </c>
       <c r="J18" t="s">
         <v>135</v>
       </c>
@@ -1785,7 +1808,7 @@
         <v>46</v>
       </c>
       <c r="M18" t="s">
-        <v>55</v>
+        <v>87</v>
       </c>
       <c r="N18" t="s">
         <v>29</v>
@@ -1794,10 +1817,57 @@
         <v>30</v>
       </c>
       <c r="P18" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>136</v>
+      </c>
+      <c r="B19" t="s">
+        <v>137</v>
+      </c>
+      <c r="C19" t="s">
+        <v>138</v>
+      </c>
+      <c r="D19" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" t="s">
+        <v>51</v>
+      </c>
+      <c r="F19" t="s">
+        <v>117</v>
+      </c>
+      <c r="G19" t="s">
         <v>95</v>
       </c>
-      <c r="Q18" t="s">
-        <v>96</v>
+      <c r="H19"/>
+      <c r="I19"/>
+      <c r="J19" t="s">
+        <v>139</v>
+      </c>
+      <c r="K19"/>
+      <c r="L19" t="s">
+        <v>46</v>
+      </c>
+      <c r="M19" t="s">
+        <v>53</v>
+      </c>
+      <c r="N19" t="s">
+        <v>29</v>
+      </c>
+      <c r="O19" t="s">
+        <v>30</v>
+      </c>
+      <c r="P19" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1833,7 +1903,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"record,visit_status,range,missing_value,date_order,reconcile"</xm:f>
+            <xm:f>"record,visit_status,future_date,range,missing_value,date_order,reconcile"</xm:f>
           </x14:formula1>
           <xm:sqref>F2:F1000</xm:sqref>
         </x14:dataValidation>
@@ -1862,7 +1932,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>6</v>
@@ -1877,7 +1947,7 @@
         <v>9</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2">
@@ -1885,137 +1955,160 @@
         <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C2" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D2" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="E2" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F2" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="G2" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B3" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C3" t="s">
+        <v>149</v>
+      </c>
+      <c r="D3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E3" t="s">
         <v>145</v>
       </c>
-      <c r="D3" t="s">
-        <v>146</v>
-      </c>
-      <c r="E3" t="s">
-        <v>141</v>
-      </c>
       <c r="F3" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="G3" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>123</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="D4" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="E4" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="F4" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="G4" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>127</v>
       </c>
       <c r="B5" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C5" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="D5" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="E5" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F5" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="G5" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>129</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="C6" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="D6" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="E6" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F6" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="G6" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>133</v>
       </c>
       <c r="B7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="C7" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E7" t="s">
+        <v>145</v>
+      </c>
+      <c r="F7" t="s">
+        <v>169</v>
+      </c>
+      <c r="G7" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B8" t="s">
+        <v>171</v>
+      </c>
+      <c r="C8" t="s">
+        <v>172</v>
+      </c>
+      <c r="D8" t="s">
         <v>156</v>
       </c>
-      <c r="E7" t="s">
-        <v>141</v>
-      </c>
-      <c r="F7" t="s">
-        <v>164</v>
-      </c>
-      <c r="G7" t="s">
-        <v>165</v>
+      <c r="E8" t="s">
+        <v>145</v>
+      </c>
+      <c r="F8" t="s">
+        <v>173</v>
+      </c>
+      <c r="G8" t="s">
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2034,37 +2127,37 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>